<commit_message>
Week 1 end : connect to Outlook and read Yucho receipt emails
Check point
◦　Authentication Flow Completed  — Microsoft accepted your login
◦　Oauth Access Token Stored  — Token saved to o365_token.txt file
◦　Connected successfully!  — Python is connected to Hotmail
</commit_message>
<xml_diff>
--- a/Procedure and Memo.xlsx
+++ b/Procedure and Memo.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\student\Desktop\Portfolio\Receipt-Automation-Pipeline\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AC80CE2-4755-40A1-BFE9-3F74CB9EC3CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C7F393-042F-4EEE-ABFD-E9D97B932687}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Procedure" sheetId="1" r:id="rId1"/>
     <sheet name="Memo" sheetId="2" r:id="rId2"/>
+    <sheet name="Troubleshooting" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -141,22 +142,22 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="82">
   <si>
     <t>created the path C:\Users\student\Desktop\Portfolio\Receipt-Automation-Pipeline</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>set up a virtual environment (python) \venv\Scripts\activate</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>added additional packet  pip install requests msal gspread google-auth streamlit pandas</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t xml:space="preserve">#pandas is installed </t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <r>
@@ -181,7 +182,7 @@
       </rPr>
       <t>: Used to send commands to a website or API (e.g., retrieving data from the web or sending data elsewhere).</t>
     </r>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <r>
@@ -206,7 +207,7 @@
       </rPr>
       <t>: (Microsoft Authentication Library) Used for logging into Microsoft systems, such as connecting to Outlook, SharePoint, or Azure.</t>
     </r>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <r>
@@ -231,7 +232,7 @@
       </rPr>
       <t>: Used specifically for reading and writing data in Google Sheets.</t>
     </r>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <r>
@@ -256,7 +257,7 @@
       </rPr>
       <t>: Used to manage Google permissions and authentication for secure access to Google Sheets or Google Drive.</t>
     </r>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <r>
@@ -281,7 +282,7 @@
       </rPr>
       <t>: Used to quickly transform Python code into beautiful web apps or dashboards (very popular in data science).</t>
     </r>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <r>
@@ -306,11 +307,11 @@
       </rPr>
       <t>: Used to manage and analyze data in tabular format (similar to Excel but works through code).</t>
     </r>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>Create project files</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>.env</t>
@@ -335,7 +336,7 @@
   </si>
   <si>
     <t>Set up the templete shows what credential are needed  in .env.example</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t># Microsoft Graph API</t>
@@ -360,7 +361,7 @@
   </si>
   <si>
     <t>Create .gitgnore to ignore .evn and venv</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>venv/</t>
@@ -402,15 +403,15 @@
       </rPr>
       <t xml:space="preserve"> คือไฟล์ที่เอาไวเก็บความลับห้ามบอกคนอื่นห้ามอัพลง เช่น </t>
     </r>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t xml:space="preserve">Password </t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>API key</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <r>
@@ -483,7 +484,7 @@
       </rPr>
       <t xml:space="preserve"> เอาไว้ให้คนอื่นดู</t>
     </r>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>GOOGLE_SHEET_ID=your_id_here</t>
@@ -493,11 +494,11 @@
   </si>
   <si>
     <t>sign in with my oamplove5@hotmail.com account.</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t xml:space="preserve">Access to Microsoft Entra by  https://entra.microsoft.com  </t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <r>
@@ -513,27 +514,27 @@
       </rPr>
       <t>การระบุตัวตนและการเข้าถึงเครือข่าย</t>
     </r>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>Told Microsoft "this script has permission to read emails from this Hotmail account". The CLIENT_ID, CLIENT_SECRET, TENANT_ID are like a username/password for your app.</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>install 0365 via powershell</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>Mail.Read  = Python can read emails</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>offline_access = Python can stay connected without logging in every time</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>Added API Permission Mail.Read &amp; offline_access. Let my app can read the email</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <r>
@@ -665,7 +666,7 @@
       </rPr>
       <t>บนคอมพิวเตอร์ของคุณ</t>
     </r>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <r>
@@ -786,11 +787,11 @@
   </si>
   <si>
     <t>Use o365 to conect Outlook for API read mail</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>dotenv fetch API Key ,Client ID, Client Secret, Database password</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <r>
@@ -860,17 +861,129 @@
       </rPr>
       <t xml:space="preserve"> .evn</t>
     </r>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>scopes</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>These are the permissions we requested from Microsoft.
 'basic' → Basic account information
 'message_all' → Access to all emails</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Real problems encountered during development and how they were solved</t>
+  </si>
+  <si>
+    <t>Problem 1 — School tenant blocked personal account</t>
+  </si>
+  <si>
+    <t>**Error:**</t>
+  </si>
+  <si>
+    <t>```</t>
+  </si>
+  <si>
+    <t>AADSTS90072: User account does not exist in tenant 'yoshida-g.ac.jp'</t>
+  </si>
+  <si>
+    <t>**Cause:** Computer was linked to school Microsoft account, so Azure</t>
+  </si>
+  <si>
+    <t>kept logging in with school account instead of personal Hotmail.</t>
+  </si>
+  <si>
+    <r>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fix:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFD3D7DE"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Opened Azure portal in Incognito browser and signed in manually with personal Hotmail account. </t>
+    </r>
+  </si>
+  <si>
+    <t>Invalid redirect URI</t>
+  </si>
+  <si>
+    <t>invalid_request: The provided value for the input parameter</t>
+  </si>
+  <si>
+    <t>'redirect_uri' is not valid</t>
+  </si>
+  <si>
+    <t>**Cause:** Used `http://localhost:8080` which works for Web apps</t>
+  </si>
+  <si>
+    <t>but not for personal Microsoft accounts.</t>
+  </si>
+  <si>
+    <t>**Fix:** Changed platform from Web to Mobile and desktop applications</t>
+  </si>
+  <si>
+    <t>in Azure Authentication settings and used:</t>
+  </si>
+  <si>
+    <t>https://login.microsoftonline.com/common/oauth2/nativeclient</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authentication is completed. O365 token is stored. Now can use API my script can now talk to  Hotmail inbox! </t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t xml:space="preserve">**Cause:** Browser was redirecting to "wrongplace" page and </t>
+  </si>
+  <si>
+    <t>the ?code= token was in a different browser tab.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">**Fix:** After login, check ALL open browser tabs for the one </t>
+  </si>
+  <si>
+    <t xml:space="preserve">containing ?code= in the address bar. Copy that full URL and </t>
+  </si>
+  <si>
+    <t>paste into terminal when prompted.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Redirect URL not capturing ?code=</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t xml:space="preserve">fetch the mail outlook and print for a test </t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>*please note I have the email box that named "Yucho" for store receive only the receipts for using debit card.</t>
+    <phoneticPr fontId="2"/>
   </si>
 </sst>
 </file>
@@ -878,13 +991,6 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="15">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Yu Gothic"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -984,6 +1090,14 @@
       <family val="2"/>
       <charset val="222"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFD3D7DE"/>
+      <name val="Yu Gothic"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1013,15 +1127,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -1297,6 +1411,398 @@
         <a:xfrm>
           <a:off x="670561" y="16459200"/>
           <a:ext cx="3901440" cy="2440283"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>89</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>427048</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>22921</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="図 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2AA55AF8-D648-FA77-1572-B0212FD71A90}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1341120" y="20345400"/>
+          <a:ext cx="3779848" cy="708721"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>106680</xdr:colOff>
+      <xdr:row>94</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>98</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="テキスト ボックス 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1277D265-4A1D-6703-2F02-7A962287AE6F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="777240" y="21640800"/>
+          <a:ext cx="4663440" cy="906780"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr kumimoji="1" lang="en-US" altLang="ja-JP" sz="1100"/>
+            <a:t>Check point</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr kumimoji="1" lang="en-US" altLang="ja-JP" sz="1100" baseline="0"/>
+            <a:t> </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" altLang="ja-JP" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Authentication Flow Completed</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="ja-JP"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ja-JP" altLang="en-US"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="ja-JP"/>
+            <a:t>— Microsoft accepted  login</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" altLang="ja-JP" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Oauth Access Token Stored</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="ja-JP"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ja-JP" altLang="en-US"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="ja-JP"/>
+            <a:t>— Token saved to </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="ja-JP" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>o365_token.txt</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="ja-JP"/>
+            <a:t> file</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" altLang="ja-JP" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Connected successfully!</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="ja-JP"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ja-JP" altLang="en-US"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="ja-JP"/>
+            <a:t>— Python is connected to your Hotmail</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr kumimoji="1" lang="ja-JP" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>41868</xdr:colOff>
+      <xdr:row>102</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>495901</xdr:colOff>
+      <xdr:row>113</xdr:row>
+      <xdr:rowOff>23234</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="図 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{030A6989-59BD-A5F6-D0CC-BE025D83E8F0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="712428" y="23492460"/>
+          <a:ext cx="3806833" cy="2362574"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>260526</xdr:colOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>113</xdr:row>
+      <xdr:rowOff>58133</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="図 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EBACFFE3-EF06-1216-8028-EBD2715D0580}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4954446" y="23553420"/>
+          <a:ext cx="3877134" cy="2336513"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>269135</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>523663</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="図 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CD758B08-68A8-A02E-4FAE-ADB748EB1DFF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7645295" y="312420"/>
+          <a:ext cx="4948448" cy="2057400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>457200</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>43662</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>412517</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>168075</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="図 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1E2DA479-776A-3BB0-C16F-BDF267C4F624}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5151120" y="6444462"/>
+          <a:ext cx="4649237" cy="1953213"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1699,7 +2205,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1719,34 +2225,34 @@
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="B3" s="3" t="e" vm="1">
+      <c r="B3" s="8" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="1"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="1">
@@ -1763,34 +2269,34 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="1"/>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:8">
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="1"/>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="1"/>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:8">
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1985,20 +2491,36 @@
       </c>
     </row>
     <row r="86" spans="1:2">
-      <c r="B86" s="9" t="s">
+      <c r="B86" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88">
         <v>11</v>
+      </c>
+      <c r="B88" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101">
+        <v>12</v>
+      </c>
+      <c r="B101" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2">
+      <c r="B102" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B3:H5"/>
   </mergeCells>
-  <phoneticPr fontId="3"/>
+  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
@@ -2014,7 +2536,7 @@
       <c r="A1">
         <v>1</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2032,12 +2554,12 @@
       <c r="A4">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2058,27 +2580,27 @@
       <c r="A8">
         <v>4</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="6" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2086,7 +2608,7 @@
       <c r="A13">
         <v>5</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>54</v>
       </c>
     </row>
@@ -2111,7 +2633,169 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3"/>
+  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{135E358C-4BFD-4CD4-ABD8-EC5636D7275B}">
+  <dimension ref="A1:B36"/>
+  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="B5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="B6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="B7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="B8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="B9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="B10" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="B11" s="9"/>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="B12" s="9"/>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15">
+        <v>2</v>
+      </c>
+      <c r="B15" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="B16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="B17" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="B18" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="B19" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="B20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="B21" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="B22" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="B24" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="B25" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="B26" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="B27" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="B28" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30">
+        <v>3</v>
+      </c>
+      <c r="B30" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="B31" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="B32" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2">
+      <c r="B34" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2">
+      <c r="B35" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2">
+      <c r="B36" t="s">
+        <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Week 1 Day 2: regex parser extracts all fields from receipt emails"
 Added parser.py
</commit_message>
<xml_diff>
--- a/Procedure and Memo.xlsx
+++ b/Procedure and Memo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\student\Desktop\Portfolio\Receipt-Automation-Pipeline\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C7F393-042F-4EEE-ABFD-E9D97B932687}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75453249-A533-428B-9D3D-EB52729041F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -142,7 +142,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="89">
   <si>
     <t>created the path C:\Users\student\Desktop\Portfolio\Receipt-Automation-Pipeline</t>
     <phoneticPr fontId="2"/>
@@ -983,6 +983,34 @@
   </si>
   <si>
     <t>*please note I have the email box that named "Yucho" for store receive only the receipts for using debit card.</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Extract data with Regex! -</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>I write parser.py — the code that reads the email body and pulls out the 5 fields we need.</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t xml:space="preserve">利用日時  </t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t xml:space="preserve">利用金額  </t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t xml:space="preserve">利用通貨  </t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t xml:space="preserve">承認番号  </t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t xml:space="preserve">利用店舗  </t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -1132,10 +1160,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -1466,15 +1494,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>106680</xdr:colOff>
-      <xdr:row>94</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:colOff>121920</xdr:colOff>
+      <xdr:row>114</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
-      <xdr:row>98</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
+      <xdr:colOff>91440</xdr:colOff>
+      <xdr:row>118</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1489,7 +1517,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="777240" y="21640800"/>
+          <a:off x="792480" y="26068020"/>
           <a:ext cx="4663440" cy="906780"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1710,6 +1738,50 @@
         <a:xfrm>
           <a:off x="4954446" y="23553420"/>
           <a:ext cx="3877134" cy="2336513"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>133164</xdr:colOff>
+      <xdr:row>121</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>290201</xdr:colOff>
+      <xdr:row>129</xdr:row>
+      <xdr:rowOff>84148</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="図 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F83065D-7972-680B-C21D-7A1A4EF0AD62}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1474284" y="27782520"/>
+          <a:ext cx="3509837" cy="1791028"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2205,7 +2277,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L126"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -2225,34 +2297,34 @@
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="B3" s="8" t="e" vm="1">
+      <c r="B3" s="9" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="1"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="1">
@@ -2514,6 +2586,44 @@
     <row r="102" spans="1:2">
       <c r="B102" t="s">
         <v>81</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120">
+        <v>13</v>
+      </c>
+      <c r="B120" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2">
+      <c r="B121" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2">
+      <c r="B122" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2">
+      <c r="B123" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2">
+      <c r="B124" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2">
+      <c r="B125" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2">
+      <c r="B126" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -2682,15 +2792,15 @@
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="8" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="B11" s="9"/>
+      <c r="B11" s="8"/>
     </row>
     <row r="12" spans="1:2">
-      <c r="B12" s="9"/>
+      <c r="B12" s="8"/>
     </row>
     <row r="15" spans="1:2">
       <c r="A15">

</xml_diff>

<commit_message>
save parsed receipts to Google Week 2 end : Sheets with duplicate detection"
outlook Yucho folder
        ↓
Python reads emails (O365)
        ↓
Regex extracts 6 fields (parser.py)
        ↓
Google Sheets stores data (sheets_writer.py)
</commit_message>
<xml_diff>
--- a/Procedure and Memo.xlsx
+++ b/Procedure and Memo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\student\Desktop\Portfolio\Receipt-Automation-Pipeline\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75453249-A533-428B-9D3D-EB52729041F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1411239A-5EA6-4C75-B9EB-08EE920F0DF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -142,7 +142,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="122">
   <si>
     <t>created the path C:\Users\student\Desktop\Portfolio\Receipt-Automation-Pipeline</t>
     <phoneticPr fontId="2"/>
@@ -1013,12 +1013,395 @@
     <t xml:space="preserve">利用店舗  </t>
     <phoneticPr fontId="2"/>
   </si>
+  <si>
+    <t>Open google sheet Add these</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>rename sheet to "Receipt Tracker"</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Data</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Time</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Store</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Amount</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Currency</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>go to google cloud "https://console.cloud.google.com"</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>create a new project nemed  "receipt-automation"</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Click "Google Sheets API" from results Click "Enable"</t>
+  </si>
+  <si>
+    <t>Click "Google Drive API" from results Click "Enable"</t>
+  </si>
+  <si>
+    <t>Enable Google Sheets API</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Enable Google Drive API</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Google Sheets API  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ทำให้เข้าถึงข้อมูล</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>Google Sheets</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ได้</t>
+    </r>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>จัดการข้อมูล</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>อ่านและเขียนค่าในเซลล์</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>เพิ่มแถว</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(Append), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>หรือลบข้อมูลในระดับช่วง</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(Range).</t>
+    </r>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <t>Google Drive API</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t xml:space="preserve"> เข้าถึง</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t xml:space="preserve"> GOOGLE DRIVE </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ได้</t>
+    </r>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>จัดการไฟล์</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>อัปโหลด</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> (Upload), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ดาวน์โหลด</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> (Download), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ค้นหา</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> (Search), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>และลบไฟล์</t>
+    </r>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Create Service Account</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>name "receipt-automation"</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Click "Service Accounts" from results</t>
+  </si>
+  <si>
+    <t>Click "+ Create Service Account"</t>
+  </si>
+  <si>
+    <t>Create a Key for the Service Account</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Click on the service account email to open it</t>
+  </si>
+  <si>
+    <t>Click the "Keys" tab at the top</t>
+  </si>
+  <si>
+    <t>Click "Add Key" → "Create new key"</t>
+  </si>
+  <si>
+    <t>Select "JSON"</t>
+  </si>
+  <si>
+    <t>Click "Create"</t>
+  </si>
+  <si>
+    <t>Share Google Sheet with the Service Account</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Change permission to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"Editor"</t>
+    </r>
+  </si>
+  <si>
+    <t>install " pip install gspread google-auth"</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t xml:space="preserve">add sheets_writer.py for write on the google sheet automaticlly </t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Run sheets_writer.py Google Sheets updated automatically</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>automation pipeline working truly</t>
+    <phoneticPr fontId="2"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1125,6 +1508,19 @@
       <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Yu Gothic"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Yu Gothic"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1495,13 +1891,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>121920</xdr:colOff>
-      <xdr:row>114</xdr:row>
+      <xdr:row>108</xdr:row>
       <xdr:rowOff>7620</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>91440</xdr:colOff>
-      <xdr:row>118</xdr:row>
+      <xdr:row>112</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1662,13 +2058,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>41868</xdr:colOff>
-      <xdr:row>102</xdr:row>
+      <xdr:row>96</xdr:row>
       <xdr:rowOff>175260</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>495901</xdr:colOff>
-      <xdr:row>113</xdr:row>
+      <xdr:row>107</xdr:row>
       <xdr:rowOff>23234</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1706,13 +2102,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>260526</xdr:colOff>
-      <xdr:row>103</xdr:row>
+      <xdr:row>97</xdr:row>
       <xdr:rowOff>7620</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>113</xdr:row>
+      <xdr:row>107</xdr:row>
       <xdr:rowOff>58133</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1750,13 +2146,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>133164</xdr:colOff>
-      <xdr:row>121</xdr:row>
+      <xdr:row>115</xdr:row>
       <xdr:rowOff>121920</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>290201</xdr:colOff>
-      <xdr:row>129</xdr:row>
+      <xdr:row>123</xdr:row>
       <xdr:rowOff>84148</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1782,6 +2178,270 @@
         <a:xfrm>
           <a:off x="1474284" y="27782520"/>
           <a:ext cx="3509837" cy="1791028"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>15240</xdr:colOff>
+      <xdr:row>128</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>135</xdr:row>
+      <xdr:rowOff>24152</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="図 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CAC0DE12-0697-6AD3-92ED-68289F95744A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="685800" y="30693360"/>
+          <a:ext cx="4427220" cy="1563392"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>106680</xdr:colOff>
+      <xdr:row>139</xdr:row>
+      <xdr:rowOff>221926</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>275309</xdr:colOff>
+      <xdr:row>148</xdr:row>
+      <xdr:rowOff>84210</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="図 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AB32E1E2-1827-6EC4-B59A-5679DBB59F85}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="777240" y="31997326"/>
+          <a:ext cx="4862549" cy="1919684"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>15241</xdr:colOff>
+      <xdr:row>162</xdr:row>
+      <xdr:rowOff>182881</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>320040</xdr:colOff>
+      <xdr:row>171</xdr:row>
+      <xdr:rowOff>154054</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="図 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B1A9FCB6-8F3E-DD63-CB78-9D236663D6DE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="685801" y="36758881"/>
+          <a:ext cx="4328159" cy="2028573"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>533401</xdr:colOff>
+      <xdr:row>172</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>533401</xdr:colOff>
+      <xdr:row>179</xdr:row>
+      <xdr:rowOff>224436</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="図 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2FE5DAA5-2F9B-B532-CC5C-3C8D4A5D6F5B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3886201" y="39448740"/>
+          <a:ext cx="3352800" cy="1695096"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>106680</xdr:colOff>
+      <xdr:row>186</xdr:row>
+      <xdr:rowOff>198120</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>586740</xdr:colOff>
+      <xdr:row>197</xdr:row>
+      <xdr:rowOff>79110</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="図 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7E2C678A-59DF-A0F7-A64E-9CEAA348DBC0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="777240" y="42717720"/>
+          <a:ext cx="5173980" cy="2395590"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>202</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>60960</xdr:colOff>
+      <xdr:row>209</xdr:row>
+      <xdr:rowOff>199022</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="図 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F937279C-1421-3A30-FBCE-8B0883699F35}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="701040" y="46352460"/>
+          <a:ext cx="5394960" cy="1623962"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2277,7 +2937,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L126"/>
+  <dimension ref="A1:L202"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -2575,55 +3235,222 @@
         <v>73</v>
       </c>
     </row>
-    <row r="101" spans="1:2">
-      <c r="A101">
+    <row r="95" spans="1:2">
+      <c r="A95">
         <v>12</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B95" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="102" spans="1:2">
-      <c r="B102" t="s">
+    <row r="96" spans="1:2">
+      <c r="B96" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="120" spans="1:2">
-      <c r="A120">
+    <row r="114" spans="1:6">
+      <c r="A114">
         <v>13</v>
       </c>
+      <c r="B114" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6">
+      <c r="B115" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6">
+      <c r="B116" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6">
+      <c r="B117" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6">
+      <c r="B118" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6">
+      <c r="B119" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6">
       <c r="B120" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="121" spans="1:2">
-      <c r="B121" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="122" spans="1:2">
-      <c r="B122" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="123" spans="1:2">
-      <c r="B123" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="124" spans="1:2">
-      <c r="B124" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="125" spans="1:2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6">
+      <c r="A125">
+        <v>14</v>
+      </c>
       <c r="B125" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="126" spans="1:2">
-      <c r="B126" t="s">
-        <v>87</v>
+        <v>89</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6">
+      <c r="B127" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6">
+      <c r="B128" t="s">
+        <v>91</v>
+      </c>
+      <c r="C128" t="s">
+        <v>92</v>
+      </c>
+      <c r="D128" t="s">
+        <v>93</v>
+      </c>
+      <c r="E128" t="s">
+        <v>94</v>
+      </c>
+      <c r="F128" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2">
+      <c r="A138">
+        <v>15</v>
+      </c>
+      <c r="B138" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2">
+      <c r="B139" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151">
+        <v>16</v>
+      </c>
+      <c r="B151" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="B153" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155">
+        <v>17</v>
+      </c>
+      <c r="B155" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2">
+      <c r="B157" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2">
+      <c r="A159">
+        <v>18</v>
+      </c>
+      <c r="B159" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="B160" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="B161" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="B162" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174">
+        <v>19</v>
+      </c>
+      <c r="B174" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="B175" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="B176" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
+      <c r="B177" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="B178" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2">
+      <c r="B179" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2">
+      <c r="A183">
+        <v>20</v>
+      </c>
+      <c r="B183" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2">
+      <c r="B184" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186">
+        <v>21</v>
+      </c>
+      <c r="B186" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2">
+      <c r="A199">
+        <v>22</v>
+      </c>
+      <c r="B199" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2">
+      <c r="A201">
+        <v>23</v>
+      </c>
+      <c r="B201" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2">
+      <c r="B202" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -2639,7 +3466,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEF3FDBC-99E4-40E5-AA7C-C0AF768B925F}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2737,9 +3564,30 @@
         <v>53</v>
       </c>
     </row>
-    <row r="17" spans="1:1">
+    <row r="17" spans="1:2">
       <c r="A17">
         <v>6</v>
+      </c>
+      <c r="B17" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="B18" s="6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19">
+        <v>7</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="B20" s="6" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Week  2 : add GitHub Actions for daily automation
code .yml to prompt github action
add more path .github/workflows/ daily_run.yml
action : run every day 9:00
</commit_message>
<xml_diff>
--- a/Procedure and Memo.xlsx
+++ b/Procedure and Memo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\student\Desktop\Portfolio\Receipt-Automation-Pipeline\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1411239A-5EA6-4C75-B9EB-08EE920F0DF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F35DA83-8019-4178-99EF-6981510E8061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -142,7 +142,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="142">
   <si>
     <t>created the path C:\Users\student\Desktop\Portfolio\Receipt-Automation-Pipeline</t>
     <phoneticPr fontId="2"/>
@@ -1396,12 +1396,638 @@
     <t>automation pipeline working truly</t>
     <phoneticPr fontId="2"/>
   </si>
+  <si>
+    <t>Github Action start!</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>GitHub Actions</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ช่วยให้คุณสามารถสั่งให้โค้ดทำงานบางอย่างโดยอัตโนมัติเมื่อเกิดเหตุการณ์</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(Events) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ต่างๆ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ใน</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Repository </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ของคุณ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Facebook
+Facebook
+ +3</t>
+    </r>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ระบบที่เอาไว้เก็บข้อมูลที่มีความสำคัญสูงหรือข้อมูลที่เป็น</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ความลับ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">" (Sensitive information) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>เช่น</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">API Keys, Passwords, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>หรือ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Tokens </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ต่างๆ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ที่เราต้องใช้ใน</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">GitHub Actions </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>แต่ไม่อยากเขียนลงไปในโค้ดตรงๆ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(Hardcode) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>เพราะจะทำให้คนอื่นเห็นได้ครับ</t>
+    </r>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ความปลอดภัย</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ข้อมูลจะถูกเข้ารหัส</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> (Encrypted) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>และจะไม่ปรากฏใน</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> Logs </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>ของ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> GitHub Actions (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>จะขึ้นเป็นเครื่องหมาย</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> *** </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t>แทน</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t xml:space="preserve">GitHub Secrets </t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>go to github &gt; repo &gt; Secrets and variables &gt; action</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t xml:space="preserve">New repository secret </t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <t>CLIENT_ID</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="222"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>&gt;  CLIENT_ID from  .env file</t>
+    </r>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>GOOGLE_SHEET_NAME &gt; Receipt Tracker</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>GOOGLE_CREDENTIALS &gt; entrie contects of google_credentials.json</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ดูวิธีเขียนโค้ดจาก &gt; https://docs.github.com/ja/actions</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t xml:space="preserve">code .yml to prompt github action </t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <t>on</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF569CD6"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>schedule</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">    - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF569CD6"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>cron</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCE9178"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>'0 0 * * *'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF6A9955"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"># Runs every day at 9:00 AM Japan time </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF569CD6"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>workflow_dispatch</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>:  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF6A9955"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t># Allows manual trigger from GitHub</t>
+    </r>
+  </si>
+  <si>
+    <t>add more path .github/workflows/ daily_run.yml</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>action : run every day 9:00</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>s</t>
+    <phoneticPr fontId="2"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1522,6 +2148,30 @@
       <family val="3"/>
       <charset val="128"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFCCCCCC"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF569CD6"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFCE9178"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF6A9955"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1543,7 +2193,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1559,6 +2209,13 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2450,6 +3107,94 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>45721</xdr:colOff>
+      <xdr:row>217</xdr:row>
+      <xdr:rowOff>140005</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>647701</xdr:colOff>
+      <xdr:row>225</xdr:row>
+      <xdr:rowOff>128229</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="図 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6E164D3E-96D1-D3AB-8200-CB74F5D3C104}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="716281" y="49746205"/>
+          <a:ext cx="5295900" cy="1817024"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>235</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>518160</xdr:colOff>
+      <xdr:row>242</xdr:row>
+      <xdr:rowOff>13207</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="図 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4B7905BB-CD36-57E6-1803-968AED4185D2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="670560" y="53263801"/>
+          <a:ext cx="5212080" cy="1613406"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2937,7 +3682,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L202"/>
+  <dimension ref="A1:L234"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -3451,6 +4196,80 @@
     <row r="202" spans="1:2">
       <c r="B202" t="s">
         <v>121</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2">
+      <c r="A212">
+        <v>24</v>
+      </c>
+      <c r="B212" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2">
+      <c r="B213" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2">
+      <c r="B214" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2">
+      <c r="B215" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2">
+      <c r="B216" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2">
+      <c r="B217" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="228" spans="1:9">
+      <c r="A228">
+        <v>25</v>
+      </c>
+      <c r="B228" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="229" spans="1:9">
+      <c r="B229" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="230" spans="1:9">
+      <c r="B230" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="231" spans="1:9">
+      <c r="B231" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="I231" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="232" spans="1:9">
+      <c r="B232" s="12" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="233" spans="1:9">
+      <c r="B233" s="12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="234" spans="1:9">
+      <c r="B234" s="12" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -3466,7 +4285,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEF3FDBC-99E4-40E5-AA7C-C0AF768B925F}">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3588,6 +4407,42 @@
     <row r="20" spans="1:2">
       <c r="B20" s="6" t="s">
         <v>105</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21">
+        <v>8</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="B22" s="10" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23">
+        <v>9</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="B24" s="6" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="B25" s="6" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="B26" s="5" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>